<commit_message>
Fase 2: actualiza Gestor SSCC a la version del 23-10
</commit_message>
<xml_diff>
--- a/Fase 2/Evidencias Proyecto/Evidencias de sistema/Aplicación/duoc/archivos de referencia/Detalle.xlsx
+++ b/Fase 2/Evidencias Proyecto/Evidencias de sistema/Aplicación/duoc/archivos de referencia/Detalle.xlsx
@@ -527,18 +527,18 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>E900019</t>
+          <t>E611658</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>EE800006</t>
+          <t>EE611658</t>
         </is>
       </c>
       <c r="C2" t="inlineStr"/>
       <c r="D2" t="inlineStr">
         <is>
-          <t>315822266</t>
+          <t>76464462K</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -569,7 +569,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>9900000055</t>
+          <t>5716095802</t>
         </is>
       </c>
       <c r="L2" t="inlineStr"/>
@@ -609,18 +609,18 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E900078</t>
+          <t>E103785</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>EE800001</t>
+          <t>EE103785</t>
         </is>
       </c>
       <c r="C3" t="inlineStr"/>
       <c r="D3" t="inlineStr">
         <is>
-          <t>317802015</t>
+          <t>773747253</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -647,7 +647,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>9900000078</t>
+          <t>8227547240</t>
         </is>
       </c>
       <c r="L3" t="inlineStr"/>
@@ -687,18 +687,18 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E900080</t>
+          <t>E602297</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>E900080</t>
+          <t>E602297</t>
         </is>
       </c>
       <c r="C4" t="inlineStr"/>
       <c r="D4" t="inlineStr">
         <is>
-          <t>321365568</t>
+          <t>785087658</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -729,7 +729,7 @@
       </c>
       <c r="K4" t="inlineStr">
         <is>
-          <t>9900000073</t>
+          <t>7462729157</t>
         </is>
       </c>
       <c r="L4" t="inlineStr"/>
@@ -769,18 +769,18 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E900121</t>
+          <t>E797122</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>E900121</t>
+          <t>E797122</t>
         </is>
       </c>
       <c r="C5" t="inlineStr"/>
       <c r="D5" t="inlineStr">
         <is>
-          <t>315109551</t>
+          <t>761410121</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -811,7 +811,7 @@
       </c>
       <c r="K5" t="inlineStr">
         <is>
-          <t>9900000088</t>
+          <t>8865815672</t>
         </is>
       </c>
       <c r="L5" t="inlineStr"/>
@@ -851,18 +851,18 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>E900045</t>
+          <t>E546405</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>EE800005</t>
+          <t>EE546405</t>
         </is>
       </c>
       <c r="C6" t="inlineStr"/>
       <c r="D6" t="inlineStr">
         <is>
-          <t>315743071</t>
+          <t>764451589</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -893,7 +893,7 @@
       </c>
       <c r="K6" t="inlineStr">
         <is>
-          <t>9900000003</t>
+          <t>1315393763</t>
         </is>
       </c>
       <c r="L6" t="inlineStr"/>
@@ -933,18 +933,18 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>E900062</t>
+          <t>E526627</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>EE800004</t>
+          <t>EE526627</t>
         </is>
       </c>
       <c r="C7" t="inlineStr"/>
       <c r="D7" t="inlineStr">
         <is>
-          <t>321444752</t>
+          <t>785172752</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -975,7 +975,7 @@
       </c>
       <c r="K7" t="inlineStr">
         <is>
-          <t>9900000091</t>
+          <t>9054925374</t>
         </is>
       </c>
       <c r="L7" t="inlineStr"/>
@@ -1015,18 +1015,18 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>E900061</t>
+          <t>E259330</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>EE800002</t>
+          <t>EE259330</t>
         </is>
       </c>
       <c r="C8" t="inlineStr"/>
       <c r="D8" t="inlineStr">
         <is>
-          <t>319623384</t>
+          <t>780131993</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="K8" t="inlineStr">
         <is>
-          <t>9900000021</t>
+          <t>2508440552</t>
         </is>
       </c>
       <c r="L8" t="inlineStr"/>
@@ -1101,18 +1101,18 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>E900063</t>
+          <t>E997738</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>EE800008</t>
+          <t>EE997738</t>
         </is>
       </c>
       <c r="C9" t="inlineStr"/>
       <c r="D9" t="inlineStr">
         <is>
-          <t>315901450</t>
+          <t>764647661</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -1143,7 +1143,7 @@
       </c>
       <c r="K9" t="inlineStr">
         <is>
-          <t>9900000045</t>
+          <t>4763341403</t>
         </is>
       </c>
       <c r="L9" t="inlineStr"/>
@@ -1183,18 +1183,18 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>E900034</t>
+          <t>E911626</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>EE800007</t>
+          <t>EE911626</t>
         </is>
       </c>
       <c r="C10" t="inlineStr"/>
       <c r="D10" t="inlineStr">
         <is>
-          <t>321999086</t>
+          <t>786435366</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -1225,7 +1225,7 @@
       </c>
       <c r="K10" t="inlineStr">
         <is>
-          <t>9900000028</t>
+          <t>3194599248</t>
         </is>
       </c>
       <c r="L10" t="inlineStr"/>
@@ -1265,18 +1265,18 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>E900100</t>
+          <t>E320303</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>EE800003</t>
+          <t>EE320303</t>
         </is>
       </c>
       <c r="C11" t="inlineStr"/>
       <c r="D11" t="inlineStr">
         <is>
-          <t>314951176</t>
+          <t>760891053</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -1307,7 +1307,7 @@
       </c>
       <c r="K11" t="inlineStr">
         <is>
-          <t>9900000002</t>
+          <t>1205468262</t>
         </is>
       </c>
       <c r="L11" t="inlineStr"/>
@@ -1559,12 +1559,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>E900019</t>
+          <t>E611658</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>9BVRG6ZD8TE900019</t>
+          <t>9BVRG6ZD8TE611658</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -1581,12 +1581,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>E900078</t>
+          <t>E103785</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>YV2RT4ZA1TE900078</t>
+          <t>YV2RT4ZA1TE103785</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
@@ -1603,12 +1603,12 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>E900080</t>
+          <t>E602297</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>YV2RT4ZA4TE900080</t>
+          <t>YV2RT4ZA4TE602297</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -1625,12 +1625,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>E900121</t>
+          <t>E797122</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>YV2XT4ZC3TE900121</t>
+          <t>YV2XT4ZC3TE797122</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -1647,12 +1647,12 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>E900045</t>
+          <t>E546405</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>9BVX20AC8TE900045</t>
+          <t>9BVX20AC8TE546405</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -1669,12 +1669,12 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>E900062</t>
+          <t>E526627</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>YV2KT4ZA8TE900062</t>
+          <t>YV2KT4ZA8TE526627</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -1691,12 +1691,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>E900061</t>
+          <t>E259330</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>YV2KG6ZB2TE900061</t>
+          <t>YV2KG6ZB2TE259330</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1713,12 +1713,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>E900063</t>
+          <t>E997738</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>YV2KT4ZB9TE900063</t>
+          <t>YV2KT4ZB9TE997738</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1735,12 +1735,12 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>E900034</t>
+          <t>E911626</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>9BVRT4ZC9TE900034</t>
+          <t>9BVRT4ZC9TE911626</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
@@ -1757,12 +1757,12 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>E900100</t>
+          <t>E320303</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>YV2XG6ZA4TE900100</t>
+          <t>YV2XG6ZA4TE320303</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">

</xml_diff>